<commit_message>
Schema 2.12 and issue log pass: solve what the data on hand allows
- PO exports dated 26 Sep 2026 from file metadata and receipt dates (D-083, D-094)
- normaliser: drop Instamart rows pasted one column left when their order exists
  correctly elsewhere; July 2025 regenerated, 59,550 -> 310 units (D-126); tests
- issue log: D-076 solved; evidence added to D-007, D-071, D-072, D-074, D-075,
  D-125; new D-127; 86 solved, 41 unsolved

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/warehouse/docs/Data_Issues_and_Doubts_Log_2026-10-30.xlsx
+++ b/warehouse/docs/Data_Issues_and_Doubts_Log_2026-10-30.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Unsolved" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Solved'!$A$1:$G$83</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Unsolved'!$A$1:$I$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Solved'!$A$1:$G$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Unsolved'!$A$1:$I$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,132 +459,139 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Solved</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Solved</t>
+          <t>Unsolved</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>82</v>
+        <v>41</v>
       </c>
       <c r="C4" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="D4" t="n">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="E4" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Unsolved</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>43</v>
-      </c>
-      <c r="C5" t="n">
-        <v>8</v>
-      </c>
-      <c r="D5" t="n">
-        <v>22</v>
-      </c>
-      <c r="E5" t="n">
         <v>13</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Unsolved by status</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Unsolved by status</t>
-        </is>
+          <t>Awaiting confirmation</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Awaiting confirmation</t>
+          <t>Open - ERP team</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Open - ERP team</t>
+          <t>Open - business</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Open - business</t>
+          <t>Parked - Blinkit</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Parked - Blinkit</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Solved: what the issue was and how it was solved (by a business answer, or handled in the warehouse).</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Solved: what the issue was and how it was solved (by a business answer, or handled in the warehouse).</t>
+          <t>Unsolved: what the issue is, the evidence, why it matters, and what is needed to close it.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Unsolved: what the issue is, the evidence, why it matters, and what is needed to close it.</t>
+          <t>Replaces Data_Issues_and_Doubts_Log_2026-10-26.xlsx (kept for history). Same IDs; D-122 to D-127 are new.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Replaces Data_Issues_and_Doubts_Log_2026-10-26.xlsx (kept for history). Same IDs; D-122 to D-125 are new.</t>
+          <t>Updated 30 Oct 2026 (second pass): issues solved from the data on hand, evidence added to open ones.</t>
         </is>
       </c>
     </row>
@@ -599,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2576,22 +2583,22 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>D-077</t>
+          <t>D-076</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Returns</t>
+          <t>Retail sales</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>One credit note can cover several goods receipts with different dates</t>
+          <t>Channels seen only in last year's returns</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Approved with Target Data Model v2 (1 Oct 2026): rule BR-023</t>
+          <t>Ellementry International = B2C export (27 Oct 2026, schema 2.8). Flipkart Website mapped to Flipkart; the old Blinkit Mumbai / Pune contacts are parked with the Blinkit data.</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
@@ -2601,44 +2608,44 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>Data team</t>
+          <t>Business (you)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>D-081</t>
+          <t>D-077</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Quick commerce</t>
+          <t>Returns</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Instamart's 'Elle SKU' shows Excel's N/A lookup error where its lookup failed</t>
+          <t>One credit note can cover several goods receipts with different dates</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Excel error values are treated as 'no SKU': rows go to Unknown and are counted</t>
+          <t>Approved with Target Data Model v2 (1 Oct 2026): rule BR-023</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>Handled in the warehouse</t>
+          <t>Resolved by the business</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -2650,22 +2657,22 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>D-082</t>
+          <t>D-081</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Returns</t>
+          <t>Quick commerce</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Return date column mixes real Excel dates and typed text</t>
+          <t>Instamart's 'Elle SKU' shows Excel's N/A lookup error where its lookup failed</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Loader stores Excel dates as ISO text and keeps typed text unchanged; staging parses both</t>
+          <t>Excel error values are treated as 'no SKU': rows go to Unknown and are counted</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -2675,7 +2682,7 @@
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -2687,22 +2694,22 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>D-084</t>
+          <t>D-082</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Returns</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>These exports carry no date of their own</t>
+          <t>Return date column mixes real Excel dates and typed text</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Loader requires --as-of for every snapshot, state or master file. When saving these exports, put the full export date in the file name</t>
+          <t>Loader stores Excel dates as ISO text and keeps typed text unchanged; staging parses both</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
@@ -2717,29 +2724,29 @@
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>Business (you)</t>
+          <t>Data team</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>D-085</t>
+          <t>D-083</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>Purchase orders</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>7 locations are selected in the report filter but have no column</t>
+          <t>The PO export's real date is unknown</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Checked against all 19 stock reports (31 Mar 2025 - 15 Sep 2026): these 7 locations never had a column, i.e. never held stock. The ERP leaves empty locations out. Nothing to fix.</t>
+          <t>Solved from the files themselves: both Pending PO files were saved on 26 Sep 2026 (file metadata, ~12:00 IST; '12.22' / '12.09' in the names are times), and the FY 25-26 file holds goods receipts up to 24 Sep 2026. Schema 2.12: both exports dated 26 Sep 2026; the 'export date assumed' label is gone.</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
@@ -2754,29 +2761,29 @@
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>ERP team</t>
+          <t>Business (you)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>D-086</t>
+          <t>D-084</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Report ends with a grand-total row</t>
+          <t>These exports carry no date of their own</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Every location column must add up to its footer total, and every row to its Total column, or the whole file is rejected</t>
+          <t>Loader requires --as-of for every snapshot, state or master file. When saving these exports, put the full export date in the file name</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
@@ -2791,29 +2798,29 @@
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>Data team</t>
+          <t>Business (you)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>D-087</t>
+          <t>D-085</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Product master</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Sheet1 also contains a full copy of stock columns</t>
+          <t>7 locations are selected in the report filter but have no column</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>Only the 5 product columns are loaded; the stock copy is ignored by design</t>
+          <t>Checked against all 19 stock reports (31 Mar 2025 - 15 Sep 2026): these 7 locations never had a column, i.e. never held stock. The ERP leaves empty locations out. Nothing to fix.</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
@@ -2828,29 +2835,29 @@
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>Data team</t>
+          <t>ERP team</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>D-088</t>
+          <t>D-086</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Quick commerce</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Columns without a header</t>
+          <t>Report ends with a grand-total row</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Dropped only after checking they are exactly a counter / only '--'; otherwise the file is rejected</t>
+          <t>Every location column must add up to its footer total, and every row to its Total column, or the whole file is rejected</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
@@ -2860,7 +2867,7 @@
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -2872,22 +2879,22 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>D-091</t>
+          <t>D-087</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Domestic sales</t>
+          <t>Product master</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Classification by elimination is unsafe until the partner list is complete</t>
+          <t>Sheet1 also contains a full copy of stock columns</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Safety switch partner_list_complete = false: unlisted names stay UNCLASSIFIED until the business confirms the list is complete</t>
+          <t>Only the 5 product columns are loaded; the stock copy is ignored by design</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
@@ -2897,7 +2904,7 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -2909,22 +2916,22 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>D-093</t>
+          <t>D-088</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Stock transfers</t>
+          <t>Quick commerce</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Inward prefix 'STK' is shared by two receiving locations</t>
+          <t>Columns without a header</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Receiver taken from the linked outward document, not from the prefix</t>
+          <t>Dropped only after checking they are exactly a counter / only '--'; otherwise the file is rejected</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
@@ -2934,7 +2941,7 @@
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -2946,27 +2953,27 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>D-095</t>
+          <t>D-091</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>Domestic sales</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Stock 'as on 31-03-2025' not yet requested; rule BR-021 ('stock history cannot be re-pulled') is out of date for ERP locations</t>
+          <t>Classification by elimination is unsafe until the partner list is complete</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Stock reports for 31 Mar 2025 and every month-end to 31 Aug 2026 received (Oct 2026). Schema 2.11: 31 Mar 2025 is the opening stock (BR-033); month-end stock trend on the Stock dashboard.</t>
+          <t>Safety switch partner_list_complete = false: unlisted names stay UNCLASSIFIED until the business confirms the list is complete</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>Resolved by the business</t>
+          <t>Handled in the warehouse</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
@@ -2976,34 +2983,34 @@
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>ERP team</t>
+          <t>Data team</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>D-096</t>
+          <t>D-093</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Quick commerce</t>
+          <t>Stock transfers</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Blinkit and Instamart stock at 15-Sep-2026 cannot be re-fetched; only current-day stock is available</t>
+          <t>Inward prefix 'STK' is shared by two receiving locations</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Accepted gap</t>
+          <t>Receiver taken from the linked outward document, not from the prefix</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>Resolved by the business</t>
+          <t>Handled in the warehouse</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
@@ -3013,34 +3020,34 @@
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>Business (you)</t>
+          <t>Data team</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>D-097</t>
+          <t>D-094</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Quick commerce</t>
+          <t>Purchase orders</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Blinkit and Instamart sales history is a manually assembled workbook and cannot be re-fetched month by month</t>
+          <t>Export date of both PO files is unknown ('12.22' and '12.09' in the file names: time or date unclear)</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Decision: originals untouched; cleaned monthly files loaded; cleaning rules still to be confirmed in CLEANING_PLAN.md</t>
+          <t>Same evidence as D-083: export date 26 Sep 2026 for both PO files (schema 2.12, MANIFEST.tsv). Overdue days on open PO lines are now measured to that date.</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>Resolved by the business</t>
+          <t>Handled in the warehouse</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
@@ -3050,178 +3057,178 @@
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>Data team</t>
+          <t>Business (you)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
+          <t>D-095</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Inventory</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Stock 'as on 31-03-2025' not yet requested; rule BR-021 ('stock history cannot be re-pulled') is out of date for ERP locations</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Stock reports for 31 Mar 2025 and every month-end to 31 Aug 2026 received (Oct 2026). Schema 2.11: 31 Mar 2025 is the opening stock (BR-033); month-end stock trend on the Stock dashboard.</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>Resolved by the business</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>ERP team</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>D-096</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Quick commerce</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Blinkit and Instamart stock at 15-Sep-2026 cannot be re-fetched; only current-day stock is available</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Accepted gap</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>Resolved by the business</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>Business (you)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>D-097</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Quick commerce</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Blinkit and Instamart sales history is a manually assembled workbook and cannot be re-fetched month by month</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Decision: originals untouched; cleaned monthly files loaded; cleaning rules still to be confirmed in CLEANING_PLAN.md</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>Resolved by the business</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>Data team</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
           <t>D-099</t>
         </is>
       </c>
-      <c r="B67" s="4" t="inlineStr">
+      <c r="B70" s="4" t="inlineStr">
         <is>
           <t>WMS dispatch</t>
         </is>
       </c>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="C70" s="4" t="inlineStr">
         <is>
           <t>Dispatch file is .xlsm and Order Date is a real Excel date, but the draft WMS_DISPATCH contract expects text</t>
         </is>
       </c>
-      <c r="D67" s="4" t="inlineStr">
+      <c r="D70" s="4" t="inlineStr">
         <is>
           <t>Contract to be corrected against the real file before loading. Ask Operations to export future dispatch reports as CSV with ID columns as text
 2026-10-22: contract verified against the full .xlsm export; dates read as real Excel date-times.</t>
         </is>
       </c>
-      <c r="E67" s="4" t="inlineStr">
+      <c r="E70" s="4" t="inlineStr">
         <is>
           <t>Handled in the warehouse</t>
         </is>
       </c>
-      <c r="F67" s="4" t="inlineStr">
+      <c r="F70" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G67" s="4" t="inlineStr">
+      <c r="G70" s="4" t="inlineStr">
         <is>
           <t>Business (you)</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>D-100</t>
-        </is>
-      </c>
-      <c r="B68" s="4" t="inlineStr">
-        <is>
-          <t>Purchase orders</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>PO reports now have an extra column 'Document Remark' (38 columns; contract has 37)</t>
-        </is>
-      </c>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>Contract updated to 38 columns (schema 2.3); the meaning of Document Remark confirmed as rule BR-031 (schema 2.10).</t>
-        </is>
-      </c>
-      <c r="E68" s="4" t="inlineStr">
-        <is>
-          <t>Resolved by the business</t>
-        </is>
-      </c>
-      <c r="F68" s="4" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G68" s="4" t="inlineStr">
-        <is>
-          <t>Data team</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="4" t="inlineStr">
-        <is>
-          <t>D-101</t>
-        </is>
-      </c>
-      <c r="B69" s="4" t="inlineStr">
-        <is>
-          <t>Product master</t>
-        </is>
-      </c>
-      <c r="C69" s="4" t="inlineStr">
-        <is>
-          <t>The first Final Master copy supplied lacked Sheet1</t>
-        </is>
-      </c>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>Original file supplied</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>Resolved by the business</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G69" s="4" t="inlineStr">
-        <is>
-          <t>Business (you)</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="4" t="inlineStr">
-        <is>
-          <t>D-102</t>
-        </is>
-      </c>
-      <c r="B70" s="4" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>Warehouse is to run on PostgreSQL 18; it was tested on PostgreSQL 16</t>
-        </is>
-      </c>
-      <c r="D70" s="4" t="inlineStr">
-        <is>
-          <t>Confirmed: 78/78 schema tests (tests/test_schema.sql) and 63/63 pytest (49 loader, 6 seed, 8 transform; 0 skipped) on PostgreSQL 18.6 + Python 3.13.15, 2026-10-16</t>
-        </is>
-      </c>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>Resolved by the business</t>
-        </is>
-      </c>
-      <c r="F70" s="4" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G70" s="4" t="inlineStr">
-        <is>
-          <t>Data team</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>D-104</t>
+          <t>D-100</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Purchase orders</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Python 3.13 used instead of the preferred 3.12</t>
+          <t>PO reports now have an extra column 'Document Remark' (38 columns; contract has 37)</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Confirmed: 78/78 schema tests (tests/test_schema.sql) and 63/63 pytest (49 loader, 6 seed, 8 transform; 0 skipped) on PostgreSQL 18.6 + Python 3.13.15, 2026-10-16; requirements.txt pinned to the tested versions (commit 3ae9cea)</t>
+          <t>Contract updated to 38 columns (schema 2.3); the meaning of Document Remark confirmed as rule BR-031 (schema 2.10).</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
@@ -3243,22 +3250,22 @@
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>D-107</t>
+          <t>D-101</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Product master</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>A database named ellementry_dw already exists on the server; it belongs to the other model's prototype</t>
+          <t>The first Final Master copy supplied lacked Sheet1</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Decision: keep ellementry_dw for the prototype evaluation; our warehouse = ellementry_warehouse</t>
+          <t>Original file supplied</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
@@ -3280,22 +3287,22 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>D-108</t>
+          <t>D-102</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Retail sales</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Control total Rs 4,22,80,208.54 was mislabelled 'retail net sales' in earlier notes</t>
+          <t>Warehouse is to run on PostgreSQL 18; it was tested on PostgreSQL 16</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Rs 4,22,80,208.54 is retail INVOICED sales excluding GST, before returns (sample period Apr-Sep 2026); net of returns dated Apr-Sep 2026 = Rs 3,69,30,320.14. Corrected in PRD-001</t>
+          <t>Confirmed: 78/78 schema tests (tests/test_schema.sql) and 63/63 pytest (49 loader, 6 seed, 8 transform; 0 skipped) on PostgreSQL 18.6 + Python 3.13.15, 2026-10-16</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
@@ -3310,39 +3317,39 @@
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>Business (you)</t>
+          <t>Data team</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>D-109</t>
+          <t>D-104</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>WMS dispatch</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>WMS Invoice No for marketplace orders (M25-, M26-, M44-...) never matches an ERP bill</t>
+          <t>Python 3.13 used instead of the preferred 3.12</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Schema 2.5: link by Invoice No, else Extern Order No = bill order number, else Tracking No = bill AWB. Linked 24,893 -&gt; 45,171 of 45,246. The M-series are the marketplaces' own invoice numbers (accounts may confirm; nothing depends on it now)</t>
+          <t>Confirmed: 78/78 schema tests (tests/test_schema.sql) and 63/63 pytest (49 loader, 6 seed, 8 transform; 0 skipped) on PostgreSQL 18.6 + Python 3.13.15, 2026-10-16; requirements.txt pinned to the tested versions (commit 3ae9cea)</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>Handled in the warehouse</t>
+          <t>Resolved by the business</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
@@ -3354,81 +3361,81 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>D-107</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Retail sales</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>ERP bill numbers restart every April (IN-1 exists in FY 25-26 and FY 26-27)</t>
+          <t>A database named ellementry_dw already exists on the server; it belongs to the other model's prototype</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Schema 2.6: a bill is its number within a financial year (bill_fy_start in the line identity); returns link to the latest bill of that number on or before the return; reconcile.py uses the same key. Fixed 2026-10-26. Retail sales Apr 2025 - Sep 2026: Rs 13.66 Cr -&gt; Rs 13.92 Cr; reconciles 28/28</t>
+          <t>Decision: keep ellementry_dw for the prototype evaluation; our warehouse = ellementry_warehouse</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>Handled in the warehouse</t>
+          <t>Resolved by the business</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>Data team</t>
+          <t>Business (you)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>D-114</t>
+          <t>D-108</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>WMS dispatch</t>
+          <t>Retail sales</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Weight over 100 kg on 85 deliveries (max 265,650)</t>
+          <t>Control total Rs 4,22,80,208.54 was mislabelled 'retail net sales' in earlier notes</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Schema 2.4: weights over 100 kg left out of v_fulfilment; WARN check shipment_weight_suspect</t>
+          <t>Rs 4,22,80,208.54 is retail INVOICED sales excluding GST, before returns (sample period Apr-Sep 2026); net of returns dated Apr-Sep 2026 = Rs 3,69,30,320.14. Corrected in PRD-001</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>Handled in the warehouse</t>
+          <t>Resolved by the business</t>
         </is>
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>Data team</t>
+          <t>Business (you)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>D-115</t>
+          <t>D-109</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
@@ -3438,128 +3445,128 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Site Location 'Ellementry International' maps to no channel</t>
+          <t>WMS Invoice No for marketplace orders (M25-, M26-, M44-...) never matches an ERP bill</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Ellementry International = B2C export (business, 27 Oct 2026). Schema 2.8: channel EXPORT_B2C, sales segment 'B2C export'. B2B exports go through Dileep.</t>
+          <t>Schema 2.5: link by Invoice No, else Extern Order No = bill order number, else Tracking No = bill AWB. Linked 24,893 -&gt; 45,171 of 45,246. The M-series are the marketplaces' own invoice numbers (accounts may confirm; nothing depends on it now)</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>Resolved by the business</t>
+          <t>Handled in the warehouse</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>Business (you)</t>
+          <t>Data team</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>D-116</t>
+          <t>D-110</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>Retail sales</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>103 trading SKUs have no MRP in any source (mostly discontinued)</t>
+          <t>ERP bill numbers restart every April (IN-1 exists in FY 25-26 and FY 26-27)</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Stock is valued at cost, not MRP (business, 27 Oct 2026). Schema 2.8: every trading SKU in stock has a cost in the ERP item master, so missing MRPs no longer affect stock value.</t>
+          <t>Schema 2.6: a bill is its number within a financial year (bill_fy_start in the line identity); returns link to the latest bill of that number on or before the return; reconcile.py uses the same key. Fixed 2026-10-26. Retail sales Apr 2025 - Sep 2026: Rs 13.66 Cr -&gt; Rs 13.92 Cr; reconciles 28/28</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>Resolved by the business</t>
+          <t>Handled in the warehouse</t>
         </is>
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>Business (you)</t>
+          <t>Data team</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>D-117</t>
+          <t>D-114</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>WMS dispatch</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Active MRP for the same SKU differs between locations</t>
+          <t>Weight over 100 kg on 85 deliveries (max 265,650)</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Business rule (27 Oct 2026): where MRPs disagree the higher one is current (prices were raised; the lower MRP is old stock). Schema 2.8 takes the highest of stock report, latest invoice and item master.</t>
+          <t>Schema 2.4: weights over 100 kg left out of v_fulfilment; WARN check shipment_weight_suspect</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>Resolved by the business</t>
+          <t>Handled in the warehouse</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>Business (you)</t>
+          <t>Data team</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>D-119</t>
+          <t>D-115</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>WMS dispatch</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Days of cover ignored stock leaving by transfer</t>
+          <t>Site Location 'Ellementry International' maps to no channel</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Schema 2.4: cover = sellable / (sales + transfers out) per day over 30 days</t>
+          <t>Ellementry International = B2C export (business, 27 Oct 2026). Schema 2.8: channel EXPORT_B2C, sales segment 'B2C export'. B2B exports go through Dileep.</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>Handled in the warehouse</t>
+          <t>Resolved by the business</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr">
@@ -3569,66 +3576,66 @@
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>Data team</t>
+          <t>Business (you)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>D-120</t>
+          <t>D-116</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Purchase orders</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Over-received PO lines (pending quantity below zero)</t>
+          <t>103 trading SKUs have no MRP in any source (mostly discontinued)</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Schema 2.4: v_purchase_order_lines.is_over_received; table on the Purchasing &amp; transfers dashboard. Purchasing may want to review the 24 lines</t>
+          <t>Stock is valued at cost, not MRP (business, 27 Oct 2026). Schema 2.8: every trading SKU in stock has a cost in the ERP item master, so missing MRPs no longer affect stock value.</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>Handled in the warehouse</t>
+          <t>Resolved by the business</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>Data team</t>
+          <t>Business (you)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>D-122</t>
+          <t>D-117</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Purchase orders</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Goods receipts have no receiving location (gap G-025)</t>
+          <t>Active MRP for the same SKU differs between locations</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Business (27 Oct 2026): all goods receipts arrive at Bagru. Rule BR-032, schema 2.9: setting goods_receipt_location = BAGRU_WH places all 4,906 receipts.</t>
+          <t>Business rule (27 Oct 2026): where MRPs disagree the higher one is current (prices were raised; the lower MRP is old stock). Schema 2.8 takes the highest of stock report, latest invoice and item master.</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
@@ -3650,42 +3657,190 @@
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
+          <t>D-119</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Inventory</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>Days of cover ignored stock leaving by transfer</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Schema 2.4: cover = sellable / (sales + transfers out) per day over 30 days</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>Handled in the warehouse</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>Data team</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>D-120</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Purchase orders</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>Over-received PO lines (pending quantity below zero)</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Schema 2.4: v_purchase_order_lines.is_over_received; table on the Purchasing &amp; transfers dashboard. Purchasing may want to review the 24 lines</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>Handled in the warehouse</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>Data team</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>D-122</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Purchase orders</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Goods receipts have no receiving location (gap G-025)</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Business (27 Oct 2026): all goods receipts arrive at Bagru. Rule BR-032, schema 2.9: setting goods_receipt_location = BAGRU_WH places all 4,906 receipts.</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>Resolved by the business</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>Business (you)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
           <t>D-123</t>
         </is>
       </c>
-      <c r="B83" s="4" t="inlineStr">
+      <c r="B86" s="4" t="inlineStr">
         <is>
           <t>Inventory</t>
         </is>
       </c>
-      <c r="C83" s="4" t="inlineStr">
+      <c r="C86" s="4" t="inlineStr">
         <is>
           <t>Stock was valued at MRP; the company values stock at cost</t>
         </is>
       </c>
-      <c r="D83" s="4" t="inlineStr">
+      <c r="D86" s="4" t="inlineStr">
         <is>
           <t>Schema 2.8: unit cost from the ERP item master (COST); stock_value_cost on the Stock and Executive dashboards (Rs 3.86 Cr on 15 Sep 2026; Rs 14.80 Cr at MRP).</t>
         </is>
       </c>
-      <c r="E83" s="4" t="inlineStr">
+      <c r="E86" s="4" t="inlineStr">
         <is>
           <t>Resolved by the business</t>
         </is>
       </c>
-      <c r="F83" s="4" t="inlineStr">
+      <c r="F86" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G83" s="4" t="inlineStr">
+      <c r="G86" s="4" t="inlineStr">
         <is>
           <t>Business (you)</t>
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>D-126</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Quick commerce</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Instamart July 2025 sales counted 59,550 units instead of 310</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Found by matching supply to sales: the 'june' sheet of the Instamart workbook has 37 July orders pasted one column to the left (SKU column missing), so the selling value landed in units. All 37 are copies of orders on the 'july' sheet. The normaliser now drops such a row only when its order exists correctly elsewhere (and stops otherwise); July 2025 regenerated: 310 units. Instamart total 65,734 -&gt; 6,494 units.</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>Handled in the warehouse</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>Data team</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G83"/>
+  <autoFilter ref="A1:G87"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3696,7 +3851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3832,12 +3987,12 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Quick commerce: focus is Instamart. How is stock supplied to Instamart (which invoice name or PO)? No invoices to any Swiggy / Instamart name were found in the ERP exports. Blinkit parked.</t>
+          <t>Likely answer from the data: Instamart is supplied through invoices to PJTJ TECHNOLOGIES PVT LTD and MOKSH ENTERPRISES PVT LTD (98% of their units are in Instamart's 43 SKUs; Apr 2025 - Sep 2026 they took ~6,030 units against ~6,180 Instamart sold). Confirm, and they become Instamart's partner accounts (sale-or-return).</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Open - business</t>
+          <t>Awaiting confirmation</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -4089,43 +4244,42 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>D-094</t>
+          <t>D-005</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Purchase orders</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Export date of both PO files is unknown ('12.22' and '12.09' in the file names: time or date unclear)</t>
+          <t>Blinkit return sheet (and Instamart's, if any) not received</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>File names end '12.22' and '12.09'; the sheets have no title row (header on row 1). PO Open Date in the 26-27 file runs to 24-Sep-2026.</t>
+          <t>Business confirmed returns are in a separate sheet</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>The PO table keeps each line's latest status, so a wrong as-of date can roll a line's status back</t>
+          <t>Quick-commerce returns missing; net sales overstated</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Needs the business and the ERP team to state the export date (and time) of each PO file (handled meanwhile: Loader requires --as-of for ERP_PURCHASE_ORDER; PO loading is blocked until the date is given
-2.4: meta.load_batch.as_of_is_assumed; the dashboard labels overdue days from the FY 25-26 export as 'export date assumed'.)</t>
+          <t>Old Blinkit data set aside: a new seller arrangement with Blinkit starts (Oct 2026). Revisit with the new data.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Open - business</t>
+          <t>Parked - Blinkit</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -4137,7 +4291,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>D-005</t>
+          <t>D-006</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -4147,27 +4301,27 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Blinkit return sheet (and Instamart's, if any) not received</t>
+          <t>No sell-out data from franchise and SIS stores</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Business confirmed returns are in a separate sheet</t>
+          <t>Only sell-in invoices exist in the ERP</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Quick-commerce returns missing; net sales overstated</t>
+          <t>Stock AI reads stock that later comes back as demand</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Old Blinkit data set aside: a new seller arrangement with Blinkit starts (Oct 2026). Revisit with the new data.</t>
+          <t>Business will work out how to extract it (handled meanwhile: Demand for these channels uses net sales after returns until sell-out arrives)</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Parked - Blinkit</t>
+          <t>Open - business</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -4184,32 +4338,32 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>D-006</t>
+          <t>D-024</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Domestic sales</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>No sell-out data from franchise and SIS stores</t>
+          <t>'Sundry Customer' is a catch-all account</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Only sell-in invoices exist in the ERP</t>
+          <t>171 lines, 21 bills, Rs 4,960 taxable; products incl. cake stand, paper bags, tissue, gift cards</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Stock AI reads stock that later comes back as demand</t>
+          <t>Default rule would treat it as an EMPLOYEE (not on business list)</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Business will work out how to extract it (handled meanwhile: Demand for these channels uses net sales after returns until sell-out arrives)</t>
+          <t>What is Sundry Customer (walk-in / cash B2B / misc)? (handled meanwhile: Held as UNCLASSIFIED until answered)</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -4231,37 +4385,37 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>D-024</t>
+          <t>D-039</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Domestic sales</t>
+          <t>Stock transfers</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>'Sundry Customer' is a catch-all account</t>
+          <t>Outward stock never received</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>171 lines, 21 bills, Rs 4,960 taxable; products incl. cake stand, paper bags, tissue, gift cards</t>
+          <t>31 of 622 outward documents wholly unreceived = 2,311 units (233 from Jun, 34 from May). CORRECTED total counting SKU lines, incl. partly received documents: 2,794 units in transit (built warehouse, verified independently)</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Default rule would treat it as an EMPLOYEE (not on business list)</t>
+          <t>Stock can disappear between locations</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>What is Sundry Customer (walk-in / cash B2B / misc)? (handled meanwhile: Held as UNCLASSIFIED until answered)</t>
+          <t>Schema 2.4 split the unreceived transfers: to Amazon FBA (receipts recorded by Amazon, not the ERP) vs own locations. Real exceptions: 1,441 units to own locations unreceived after 60 days; warehouse team to check (list on the Purchasing &amp; transfers dashboard).</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Open - business</t>
+          <t>Open - ERP team</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -4271,39 +4425,39 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Business (you)</t>
+          <t>ERP team</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>D-039</t>
+          <t>D-047</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Stock transfers</t>
+          <t>Purchase orders</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Outward stock never received</t>
+          <t>CORRECTED: one GRN per PO line was assumed; part deliveries list several receipts in ONE cell</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>31 of 622 outward documents wholly unreceived = 2,311 units (233 from Jun, 34 from May). CORRECTED total counting SKU lines, incl. partly received documents: 2,794 units in transit (built warehouse, verified independently)</t>
+          <t>Found by the first transform run: 47 PO lines list 155 receipts in GRNNUM (e.g. 'JPR/GRN/199;305;89') with one date and one total quantity. The loader's uniqueness check could not catch it: it is one cell, not several rows</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Stock can disappear between locations</t>
+          <t>Per-receipt dates and quantities unknown; supplier lead time approximate for those lines</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Schema 2.4 split the unreceived transfers: to Amazon FBA (receipts recorded by Amazon, not the ERP) vs own locations. Real exceptions: 1,441 units to own locations unreceived after 60 days; warehouse team to check (list on the Purchasing &amp; transfers dashboard).</t>
+          <t>Still needed: a GRN register (one row per receipt with its own date and quantity). Without it, receipts land on one date per PO line, which makes month-to-month stock checks at Bagru swing (gap G-027).</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -4325,37 +4479,37 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>D-047</t>
+          <t>D-050</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Purchase orders</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>CORRECTED: one GRN per PO line was assumed; part deliveries list several receipts in ONE cell</t>
+          <t>Same Blinkit stock reported by the ERP and by Blinkit</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Found by the first transform run: 47 PO lines list 155 receipts in GRNNUM (e.g. 'JPR/GRN/199;305;89') with one date and one total quantity. The loader's uniqueness check could not catch it: it is one cell, not several rows</t>
+          <t>'27 Blinkit - Pune P2' (ERP) and 'Pune P2 - Feeder' (Blinkit)</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Per-receipt dates and quantities unknown; supplier lead time approximate for those lines</t>
+          <t>Stock double-counted</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Still needed: a GRN register (one row per receipt with its own date and quantity). Without it, receipts land on one date per PO line, which makes month-to-month stock checks at Bagru swing (gap G-027).</t>
+          <t>Old Blinkit data set aside (new seller arrangement). Revisit with the new data.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Open - ERP team</t>
+          <t>Parked - Blinkit</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -4365,14 +4519,14 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>ERP team</t>
+          <t>Business (you)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>D-050</t>
+          <t>D-051</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -4382,27 +4536,27 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Same Blinkit stock reported by the ERP and by Blinkit</t>
+          <t>Negative 'Net scheduled inventory' values</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>'27 Blinkit - Pune P2' (ERP) and 'Pune P2 - Feeder' (Blinkit)</t>
+          <t>e.g. -92, -125</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Stock double-counted</t>
+          <t>Wrong stock at Blinkit</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Old Blinkit data set aside (new seller arrangement). Revisit with the new data.</t>
+          <t>Being confirmed with Blinkit (handled meanwhile: Stored; excluded from all stock metrics)</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Parked - Blinkit</t>
+          <t>Open - business</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -4419,7 +4573,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>D-051</t>
+          <t>D-052</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -4429,22 +4583,23 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Negative 'Net scheduled inventory' values</t>
+          <t>Amazon's own FBA inventory report not provided</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>e.g. -92, -125</t>
+          <t>FBA stock known only from the ERP</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Wrong stock at Blinkit</t>
+          <t>ERP and Amazon may disagree (see unreceived FBA transfers)</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Being confirmed with Blinkit (handled meanwhile: Stored; excluded from all stock metrics)</t>
+          <t>Can the Amazon FBA inventory report be exported?
+2026-10-22: FBA stock on dashboards is the ERP's view only; transfers to FBA shown apart as 'receipt recorded by Amazon'. (handled meanwhile: FBA locations use ERP until an Amazon report is added)</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -4466,38 +4621,37 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>D-052</t>
+          <t>D-060</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>WMS dispatch</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Amazon's own FBA inventory report not provided</t>
+          <t>Long numbers exported in scientific notation</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>FBA stock known only from the ERP</t>
+          <t>Ext Manifest No '1.60396E+13'</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>ERP and Amazon may disagree (see unreceived FBA transfers)</t>
+          <t>Digits permanently lost; IDs don't match</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Can the Amazon FBA inventory report be exported?
-2026-10-22: FBA stock on dashboards is the ERP's view only; transfers to FBA shown apart as 'receipt recorded by Amazon'. (handled meanwhile: FBA locations use ERP until an Amazon report is added)</t>
+          <t>Export IDs as text or the report as CSV (handled meanwhile: All IDs loaded as text)</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Open - business</t>
+          <t>Open - ERP team</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -4507,44 +4661,44 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Business (you)</t>
+          <t>ERP team</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>D-060</t>
+          <t>D-071</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>WMS dispatch</t>
+          <t>Locations</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Long numbers exported in scientific notation</t>
+          <t>13 ERP locations hold zero stock, incl. 7 stores with no retail invoices</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Ext Manifest No '1.60396E+13'</t>
+          <t>Stores: GK Store, Indiranagar, VR Mall, Infiniti Malad, SIB Bandra, Goa Anjuna, CG Road. Also DEPL Delhi / Lucknow / Mumbai PPOB and FBA BLR5, NAG1, DED5</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Digits permanently lost; IDs don't match</t>
+          <t>Closed locations clutter reports; stock appearing there later goes unnoticed</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Export IDs as text or the report as CSV (handled meanwhile: All IDs loaded as text)</t>
+          <t>Answered from the 19 stock reports and sales (please confirm): DEPL Lucknow held stock to Feb 2026, last sale Jan 2026 (closed ~Mar 2026); CG Road stock to Aug 2025, last sale Apr 2025; FBA DED5 used Sep-Nov 2025 only; DEPL Delhi and Mumbai PPOB billed sales to Aug 2025 but never held stock (billing points); the other locations never held stock. Confirm, and the closing dates go into the location master.</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Open - ERP team</t>
+          <t>Awaiting confirmation</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -4554,14 +4708,14 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>ERP team</t>
+          <t>Business (you)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>D-071</t>
+          <t>D-072</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -4571,27 +4725,27 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>13 ERP locations hold zero stock, incl. 7 stores with no retail invoices</t>
+          <t>'Dileep Essentials Pvt Ltd Bagru' is a different location from the Bagru warehouse</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Stores: GK Store, Indiranagar, VR Mall, Infiniti Malad, SIB Bandra, Goa Anjuna, CG Road. Also DEPL Delhi / Lucknow / Mumbai PPOB and FBA BLR5, NAG1, DED5</t>
+          <t>Uses transfer prefix BAG/ (2 documents); the Bagru warehouse uses JPR/</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Closed locations clutter reports; stock appearing there later goes unnoticed</t>
+          <t>Stock moved to / from it assigned to the wrong place</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>See 'Open questions' in Reference_Mappings_Draft_v1 (handled meanwhile: Proposed inactive; any stock or sale at an inactive location raises a warning)</t>
+          <t>Tested on the stock history: it is NOT the Bagru Popup (the Popup shows no unexplained stock in the months of these transfers). Which location is it?</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Awaiting confirmation</t>
+          <t>Open - business</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -4608,7 +4762,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>D-072</t>
+          <t>D-073</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -4618,22 +4772,22 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>'Dileep Essentials Pvt Ltd Bagru' is a different location from the Bagru warehouse</t>
+          <t>'08 Essential - DFAL' holds stock but its purpose is unknown</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Uses transfer prefix BAG/ (2 documents); the Bagru warehouse uses JPR/</t>
+          <t>688 units of 15 SKUs; transfer prefixes IS/DF and RC/DF</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Stock moved to / from it assigned to the wrong place</t>
+          <t>Stock counted as sellable when it may not be</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Is it '08 Bagru Popup'? (handled meanwhile: Left unmapped (goes to Unknown) until answered)</t>
+          <t>What is DFAL, and is its stock sellable? (handled meanwhile: Proposed not sellable until confirmed)</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -4655,32 +4809,32 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>D-073</t>
+          <t>D-079</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Locations</t>
+          <t>Returns</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>'08 Essential - DFAL' holds stock but its purpose is unknown</t>
+          <t>A return 'reason' column exists but is never filled</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>688 units of 15 SKUs; transfer prefixes IS/DF and RC/DF</t>
+          <t>Empty on all 5,924 rows</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Stock counted as sellable when it may not be</t>
+          <t>Return reasons unknown, though the ERP can hold them</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>What is DFAL, and is its stock sellable? (handled meanwhile: Proposed not sellable until confirmed)</t>
+          <t>Can the team start filling the reason when raising a credit note? Gap G-009 (handled meanwhile: Reason dimension ready; reasons load as soon as the field is filled)</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -4702,37 +4856,37 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>D-079</t>
+          <t>D-092</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Returns</t>
+          <t>Quick commerce</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>A return 'reason' column exists but is never filled</t>
+          <t>Two possible supply routes to Blinkit</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Empty on all 5,924 rows</t>
+          <t>Kiranakart (Blinkit) appears on domestic credit notes, while stock also reaches Blinkit feeder locations by ERP stock transfer</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Return reasons unknown, though the ERP can hold them</t>
+          <t>Blinkit stock split across two pools or counted twice</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Can the team start filling the reason when raising a credit note? Gap G-009 (handled meanwhile: Reason dimension ready; reasons load as soon as the field is filled)</t>
+          <t>Old Blinkit data set aside (new seller arrangement). Revisit with the new data.</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Open - business</t>
+          <t>Parked - Blinkit</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -4749,38 +4903,37 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>D-083</t>
+          <t>D-103</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Purchase orders</t>
+          <t>Product master</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>The PO export's real date is unknown</t>
+          <t>Final Master as-of date not stated in the file</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>File name says '12_09' but it has 77 POs opened after 12-Sep, the latest on 24-Sep, and receipts to 24-Sep</t>
+          <t>File metadata (docProps/core.xml): modified 2026-09-25T09:22:05Z, created 2026-02-06T11:10:55Z</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>PO state recorded against the wrong date; pending-PO view wrong</t>
+          <t>Loader requires --as-of for PRODUCT_MASTER; a wrong date mis-times SKU status (Continued / Discontinued)</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>On what date was this PO report exported? Please note the export date for every future PO pull (handled meanwhile: Loader refuses a PO file whose as-of date is earlier than dates inside it
-2.4: open PO lines from an export with an assumed date are labelled 'Overdue (export date assumed)' on the dashboard.)</t>
+          <t>See 'How the warehouse handles it now' (handled meanwhile: as_of_date 2026-09-25 used in MANIFEST.tsv, assumed from file metadata)</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Open - business</t>
+          <t>Awaiting confirmation</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -4797,37 +4950,37 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>D-092</t>
+          <t>D-105</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Quick commerce</t>
+          <t>Returns</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Two possible supply routes to Blinkit</t>
+          <t>Amazon FBA customer returns report found; candidate source that may close gap G-009 (return reasons)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Kiranakart (Blinkit) appears on domestic credit notes, while stock also reaches Blinkit feeder locations by ERP stock transfer</t>
+          <t>CSV, 12 columns incl. return-date, order-id, sku, asin, reason, detailed-disposition, customer-comments; 3,499 rows, return-date 2025-04-01 to 2026-09-14. G-009 (OPEN) names marketplace return reports as a way to fill return reasons</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Blinkit stock split across two pools or counted twice</t>
+          <t>Return reasons stay unknown for Amazon returns; the free-text customer-comments column may hold personal data</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Old Blinkit data set aside (new seller arrangement). Revisit with the new data.</t>
+          <t>See 'How the warehouse handles it now' (handled meanwhile: Not a registered source; stored in C:\ellementry_data\full\_UNREGISTERED\AMAZON_CUSTOMER_RETURNS\ and listed in MANIFEST.tsv as UNREGISTERED. Registering it needs a contract and a decision on customer-comments (exclude or restrict))</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Parked - Blinkit</t>
+          <t>Open - business</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -4844,32 +4997,32 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>D-103</t>
+          <t>D-106</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Product master</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Final Master as-of date not stated in the file</t>
+          <t>As-of dates of snapshot / master files assumed from file save times</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>File metadata (docProps/core.xml): modified 2026-09-25T09:22:05Z, created 2026-02-06T11:10:55Z</t>
+          <t>Blinkit inventory: last saved 2026-09-25T10:08:47Z (15:38 IST); tests/sample_manifest.tsv said 2026-09-26. Instamart inventory: last saved 2026-09-26T06:03:19Z (11:33 IST), matches 2026-09-26. Final Master: last saved 2026-09-25T09:22:05Z; 2026-09-15 in sample_manifest was a placeholder (owner)</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Loader requires --as-of for PRODUCT_MASTER; a wrong date mis-times SKU status (Continued / Discontinued)</t>
+          <t>Loader requires --as-of; a wrong date places stock or SKU status on the wrong day</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>See 'How the warehouse handles it now' (handled meanwhile: as_of_date 2026-09-25 used in MANIFEST.tsv, assumed from file metadata)</t>
+          <t>See 'How the warehouse handles it now' (handled meanwhile: MANIFEST.tsv as_of_date: Blinkit inventory 2026-09-25, Instamart inventory 2026-09-26, Final Master 2026-09-25 (stock files show stock at download time))</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -4891,32 +5044,32 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>D-105</t>
+          <t>D-112</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Returns</t>
+          <t>WMS dispatch</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Amazon FBA customer returns report found; candidate source that may close gap G-009 (return reasons)</t>
+          <t>RTO is recorded only for website orders</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>CSV, 12 columns incl. return-date, order-id, sku, asin, reason, detailed-disposition, customer-comments; 3,499 rows, return-date 2025-04-01 to 2026-09-14. G-009 (OPEN) names marketplace return reports as a way to fill return reasons</t>
+          <t>1,945 RTO deliveries, all website (7.9%); Amazon 3 of 9,482, others 0. Marketplace returns-to-origin are handled by the marketplace</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Return reasons stay unknown for Amazon returns; the free-text customer-comments column may hold personal data</t>
+          <t>An all-channel RTO rate (4.3%) understates the real rate and shows marketplaces as perfect</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>See 'How the warehouse handles it now' (handled meanwhile: Not a registered source; stored in C:\ellementry_data\full\_UNREGISTERED\AMAZON_CUSTOMER_RETURNS\ and listed in MANIFEST.tsv as UNREGISTERED. Registering it needs a contract and a decision on customer-comments (exclude or restrict))</t>
+          <t>The WMS dispatch report is the OMS report (business, Oct 2026), so it has nothing more. Marketplace RTO must come from seller-panel return / RTO reports (Amazon, Myntra, Tata Cliq, Nykaa).</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -4938,37 +5091,37 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>D-106</t>
+          <t>D-113</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>WMS dispatch</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>As-of dates of snapshot / master files assumed from file save times</t>
+          <t>No delivery dates for Nykaa, FNP and Flipkart</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Blinkit inventory: last saved 2026-09-25T10:08:47Z (15:38 IST); tests/sample_manifest.tsv said 2026-09-26. Instamart inventory: last saved 2026-09-26T06:03:19Z (11:33 IST), matches 2026-09-26. Final Master: last saved 2026-09-25T09:22:05Z; 2026-09-15 in sample_manifest was a placeholder (owner)</t>
+          <t>Nykaa 2,701 of 2,784 stuck at SHIPPED; FNP and Flipkart all</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Loader requires --as-of; a wrong date places stock or SKU status on the wrong day</t>
+          <t>Delivery time and late-delivery measures wrong for these channels</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>See 'How the warehouse handles it now' (handled meanwhile: MANIFEST.tsv as_of_date: Blinkit inventory 2026-09-25, Instamart inventory 2026-09-26, Final Master 2026-09-25 (stock files show stock at download time))</t>
+          <t>4,778 deliveries stuck at 'Shipped' (Nykaa 2,701, website 951, Amazon 688, Tata Cliq 208, others); 2,932 with no delivery date at all. Need: courier exports by AWB (Delhivery / Shiprocket portals) for the website, seller-panel order reports for marketplaces.</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Awaiting confirmation</t>
+          <t>Open - business</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -4985,37 +5138,37 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>D-112</t>
+          <t>D-124</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>WMS dispatch</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>RTO is recorded only for website orders</t>
+          <t>Stock moves at Bagru with no document in the exports</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>1,945 RTO deliveries, all website (7.9%); Amazon 3 of 9,482, others 0. Marketplace returns-to-origin are handled by the marketplace</t>
+          <t>Month-by-month check (schema 2.11, mart.v_stock_movement_check): over 1 Apr 2025 - 15 Sep 2026, 71,350 units arrived at Bagru and 55,188 left with no sale, transfer, return or PO receipt. E.g. Gaudeep gold diya set of 11: 9,868 arrived with no receipt; gift boxes and paper bags left with no document. List: reports/bagru_unexplained_stock.csv</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>An all-channel RTO rate (4.3%) understates the real rate and shows marketplaces as perfect</t>
+          <t>Stock between month-ends cannot be rebuilt exactly; purchases without a PO, gift-set assembly and packaging use are invisible</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>The WMS dispatch report is the OMS report (business, Oct 2026), so it has nothing more. Marketplace RTO must come from seller-panel return / RTO reports (Amazon, Myntra, Tata Cliq, Nykaa).</t>
+          <t>An item-wise stock ledger (or GRN register incl. non-PO purchases, assembly / kitting register, stock adjustment / consumption register) for Bagru, 1 Apr 2025 - 15 Sep 2026. The 'Item Wise Pending Purchase Order Tracking' file received 30 Oct 2026 was empty (01/04/2024 - 31/03/2025) and is PO-only.</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Open - business</t>
+          <t>Open - ERP team</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -5025,39 +5178,39 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Business (you)</t>
+          <t>ERP team</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>D-113</t>
+          <t>D-125</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>WMS dispatch</t>
+          <t>Quick commerce</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>No delivery dates for Nykaa, FNP and Flipkart</t>
+          <t>No Instamart inventory, and the seller portal shows only today's stock</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Nykaa 2,701 of 2,784 stuck at SHIPPED; FNP and Flipkart all</t>
+          <t>Instamart seller login gives the current day's inventory only; no official history download or API found</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Delivery time and late-delivery measures wrong for these channels</t>
+          <t>No Instamart stock or cover on the dashboards</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>4,778 deliveries stuck at 'Shipped' (Nykaa 2,701, website 951, Amazon 688, Tata Cliq 208, others); 2,932 with no delivery date at all. Need: courier exports by AWB (Delhivery / Shiprocket portals) for the website, seller-panel order reports for marketplaces.</t>
+          <t>1) Download the inventory every day from now into exports/_inbox/ (loader ready). 2) If PJTJ Technologies and Moksh Enterprises are confirmed as Instamart's buying accounts (D-007), past Instamart stock can be rebuilt as units invoiced to them minus units Instamart sold (daily sell-out on hand).</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -5079,79 +5232,79 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>D-124</t>
+          <t>D-015</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>Retail sales</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Stock moves at Bagru with no document in the exports</t>
+          <t>Two Nykaa names: 'Nykaa Fashion' (900 lines) and 'Nykaa' (34 lines)</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Month-by-month check (schema 2.11, mart.v_stock_movement_check): over 1 Apr 2025 - 15 Sep 2026, 71,350 units arrived at Bagru and 55,188 left with no sale, transfer, return or PO receipt. E.g. Gaudeep gold diya set of 11: 9,868 arrived with no receipt; gift boxes and paper bags left with no document. List: reports/bagru_unexplained_stock.csv</t>
+          <t>Payment modes 'Prepaid - Nykaa Fashion' and 'Prepaid - Nykaa'</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Stock between month-ends cannot be rebuilt exactly; purchases without a PO, gift-set assembly and packaging use are invisible</t>
+          <t>Nykaa split across two channels</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>An item-wise stock ledger (or GRN register incl. non-PO purchases, assembly / kitting register, stock adjustment / consumption register) for Bagru, 1 Apr 2025 - 15 Sep 2026. The 'Item Wise Pending Purchase Order Tracking' file received 30 Oct 2026 was empty (01/04/2024 - 31/03/2025) and is PO-only.</t>
+          <t>See 'How the warehouse handles it now' (handled meanwhile: Proposed: one channel 'Nykaa' with the two names kept as sub-channels)</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Open - ERP team</t>
+          <t>Awaiting confirmation</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>ERP team</t>
+          <t>Business (you)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>D-125</t>
+          <t>D-027</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Quick commerce</t>
+          <t>Domestic sales</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>No Instamart inventory, and the seller portal shows only today's stock</t>
+          <t>Direct export rows to Singapore, although exports are said to go through Dileep</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Instamart seller login gives the current day's inventory only; no official history download or API found</t>
+          <t>2 lines to 'Hindustan Exports', Rs 1 each</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>No Instamart stock or cover on the dashboards</t>
+          <t>Unclear classification</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>1) Download the inventory every day from now into exports/_inbox/ (loader ready). 2) Ask the Instamart category manager for a historical inventory dump. 3) Tell us how Instamart is supplied, so history can be rebuilt from shipments and the daily sell-out we already have.</t>
+          <t>Are these samples to an exporter? (handled meanwhile: Held as EXPORT_CUSTOMER; Rs 1 lines also fall under the near-free issue)</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -5161,7 +5314,7 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
@@ -5173,37 +5326,37 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>D-015</t>
+          <t>D-036</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Retail sales</t>
+          <t>Returns</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Two Nykaa names: 'Nykaa Fashion' (900 lines) and 'Nykaa' (34 lines)</t>
+          <t>Domestic returns have no clear link to the original invoice</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Payment modes 'Prepaid - Nykaa Fashion' and 'Prepaid - Nykaa'</t>
+          <t>BILLNUM here is the credit note; RTNFROMCUST is the goods receipt</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Nykaa split across two channels</t>
+          <t>Cannot compute return rate per original B2B invoice</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>See 'How the warehouse handles it now' (handled meanwhile: Proposed: one channel 'Nykaa' with the two names kept as sub-channels)</t>
+          <t>Is the original invoice number stored anywhere in this report? (handled meanwhile: Original bill kept nullable)</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Awaiting confirmation</t>
+          <t>Open - ERP team</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -5213,44 +5366,44 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Business (you)</t>
+          <t>ERP team</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>D-027</t>
+          <t>D-069</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Domestic sales</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Direct export rows to Singapore, although exports are said to go through Dileep</t>
+          <t>Currency and timezone never explicitly confirmed</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>2 lines to 'Hindustan Exports', Rs 1 each</t>
+          <t>All data appears Indian (INR, IST)</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Unclear classification</t>
+          <t>Wrong if any foreign-currency data exists</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Are these samples to an exporter? (handled meanwhile: Held as EXPORT_CUSTOMER; Rs 1 lines also fall under the near-free issue)</t>
+          <t>See 'How the warehouse handles it now' (handled meanwhile: INR and IST stored as settings)</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Open - business</t>
+          <t>Awaiting confirmation</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
@@ -5267,37 +5420,37 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>D-036</t>
+          <t>D-074</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Returns</t>
+          <t>Locations</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Domestic returns have no clear link to the original invoice</t>
+          <t>Jaipur Meeraki holds stock but has no retail invoices</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>BILLNUM here is the credit note; RTNFROMCUST is the goods receipt</t>
+          <t>145 units; no Retail Sales rows Apr-Sep 2026</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Cannot compute return rate per original B2B invoice</t>
+          <t>Store type unclear (own / SIS / franchise)</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Is the original invoice number stored anywhere in this report? (handled meanwhile: Original bill kept nullable)</t>
+          <t>From the data: Meeraki invoiced as 'Dileep Essentials Pvt Ltd Jaipur Store' until 16 Jun 2025 (300 lines) and has held stock in every report since. Is it an own store that stopped billing in Jun 2025?</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Open - ERP team</t>
+          <t>Awaiting confirmation</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -5307,39 +5460,39 @@
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>ERP team</t>
+          <t>Business (you)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>D-069</t>
+          <t>D-075</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Locations</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Currency and timezone never explicitly confirmed</t>
+          <t>Two store names don't match any ERP location</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>All data appears Indian (INR, IST)</t>
+          <t>'Dileep Essentials Pvt Ltd Jaipur Store' (7 returns) and 'Dileep Essentials Pvt Ltd Lucknow'</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Wrong if any foreign-currency data exists</t>
+          <t>Returns received at an unknown location</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>See 'How the warehouse handles it now' (handled meanwhile: INR and IST stored as settings)</t>
+          <t>The evidence-based mappings hold on the stock history: 'Jaipur Store' -&gt; Jaipur Meeraki (billing stops Jun 2025, as in D-074); 'Lucknow' -&gt; DEPL Lucknow (stock to Feb 2026, sales to Jan 2026). Please confirm.</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -5361,37 +5514,37 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>D-074</t>
+          <t>D-078</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Locations</t>
+          <t>Returns</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Jaipur Meeraki holds stock but has no retail invoices</t>
+          <t>Receipt date list shorter than the receipt list on some credit notes</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>145 units; no Retail Sales rows Apr-Sep 2026</t>
+          <t>e.g. 3 receipts with 2 dates; 100 receipts in the sample cannot be paired with a date</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Store type unclear (own / SIS / franchise)</t>
+          <t>Wrong receipt dates if paired by position</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>What kind of store is Meeraki? (handled meanwhile: Proposed own store)</t>
+          <t>Why does the ERP drop a date when several receipts share one credit note? (handled meanwhile: Unpaired receipts left out of the receipts bridge; the return uses only the dates given)</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Open - business</t>
+          <t>Open - ERP team</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -5401,39 +5554,39 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Business (you)</t>
+          <t>ERP team</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>D-075</t>
+          <t>D-090</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Locations</t>
+          <t>Domestic sales</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Two store names don't match any ERP location</t>
+          <t>'DILEEP ESSENTIALS INC' appears as a return counterparty</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>'Dileep Essentials Pvt Ltd Jaipur Store' (7 returns) and 'Dileep Essentials Pvt Ltd Lucknow'</t>
+          <t>1 row</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Returns received at an unknown location</t>
+          <t>Unclear whether it is a group export entity</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Which locations are these? (handled meanwhile: Left unmapped until answered)</t>
+          <t>What is Dileep Essentials Inc? (handled meanwhile: Listed as UNCLASSIFIED so it is never classified by elimination)</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -5455,37 +5608,37 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>D-076</t>
+          <t>D-098</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Retail sales</t>
+          <t>Domestic sales</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Channels seen only in last year's returns</t>
+          <t>DOCID is a 19-digit number stored as a number, so its last digits cannot be exact</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>'Flipkart Website', 'Ellementry International', and Blinkit Mumbai / Pune contacts</t>
+          <t>All 25,863 DOCID values (20,612 + 5,251) are 19 digits and stored as floating-point numbers (about 15-16 digits are exact)</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Channel list incomplete for FY25-26</t>
+          <t>DOCID cannot be used as a reliable key</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Which channel is 'Ellementry International'? (handled meanwhile: Flipkart and Blinkit mapped (proposed); Ellementry International left unmapped)</t>
+          <t>Ask the ERP team for a text export when convenient (handled meanwhile: DOCID is kept in the raw layer only; not used by the warehouse)</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Open - business</t>
+          <t>Open - ERP team</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
@@ -5495,44 +5648,44 @@
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Business (you)</t>
+          <t>ERP team</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>D-078</t>
+          <t>D-111</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Returns</t>
+          <t>WMS dispatch</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Receipt date list shorter than the receipt list on some credit notes</t>
+          <t>39 courier spellings for about 10 companies (Delhivery 13 ways, Bluedart 6, Ekart 4; codes ATS, XC, DL, DE_*, BD_*, EK_*)</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>e.g. 3 receipts with 2 dates; 100 receipts in the sample cannot be paired with a date</t>
+          <t>Transporter / Ext Transporter Name columns</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Wrong receipt dates if paired by position</t>
+          <t>Courier comparisons split one company across many rows</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Why does the ERP drop a date when several receipts share one credit note? (handled meanwhile: Unpaired receipts left out of the receipts bridge; the return uses only the dates given)</t>
+          <t>Confirm the courier codes: ATS = Amazon Shipping, XC = Xpressbees, DL / DLV / DE_* = Delhivery, BD_* = Blue Dart, EK_* = Ekart (all mapped from data evidence, unconfirmed).</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Open - ERP team</t>
+          <t>Awaiting confirmation</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
@@ -5542,39 +5695,39 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>ERP team</t>
+          <t>Business (you)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>D-090</t>
+          <t>D-118</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Domestic sales</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>'DILEEP ESSENTIALS INC' appears as a return counterparty</t>
+          <t>Negative stock in the ERP report</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>1 row</t>
+          <t>Jaipur C-Scheme -10, Bangalore 7 -2 units</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Unclear whether it is a group export entity</t>
+          <t>Stock totals slightly off; signals booking errors</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>What is Dileep Essentials Inc? (handled meanwhile: Listed as UNCLASSIFIED so it is never classified by elimination)</t>
+          <t>An ERP glitch the ERP team cannot fix yet; the business is looking at it. 15 Sep 2026 report, sheet ChannelwiseStock: row 1602 coll003-1 Gift card at 08 Jaipur - C-Scheme -10; row 1673 GSTEA1905 at 29 FBA WH - Bangalore 7 -1; row 3030 SWETA2778 at 29 FBA WH - Bangalore 7 -1 (32 negative rows across the 19 reports). Decide: treat as 0, exclude, or show as reported (current).</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -5589,39 +5742,39 @@
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Business (you)</t>
+          <t>ERP team</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>D-098</t>
+          <t>D-121</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Domestic sales</t>
+          <t>Purchase orders</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>DOCID is a 19-digit number stored as a number, so its last digits cannot be exact</t>
+          <t>PO lines with no due date</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>All 25,863 DOCID values (20,612 + 5,251) are 19 digits and stored as floating-point numbers (about 15-16 digits are exact)</t>
+          <t>223 lines (3 still open)</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>DOCID cannot be used as a reliable key</t>
+          <t>Cannot be judged overdue</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Ask the ERP team for a text export when convenient (handled meanwhile: DOCID is kept in the raw layer only; not used by the warehouse)</t>
+          <t>Fill due dates in the ERP (handled meanwhile: Schema 2.4: due_status 'No due date' on open PO lines)</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -5643,32 +5796,32 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>D-111</t>
+          <t>D-127</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>WMS dispatch</t>
+          <t>Stock transfers</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>39 courier spellings for about 10 companies (Delhivery 13 ways, Bluedart 6, Ekart 4; codes ATS, XC, DL, DE_*, BD_*, EK_*)</t>
+          <t>Transfers out of Bagru received by the bare name 'Dileep Essentials Pvt Ltd'</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Transporter / Ext Transporter Name columns</t>
+          <t>121 inward lines, 1,929 units (Apr - Aug 2025), sent from Bagru, receiver named only 'Dileep Essentials Pvt Ltd' (no location); Bagru shows +2,625 unexplained units of the same SKUs in the same months</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Courier comparisons split one company across many rows</t>
+          <t>These units sit at an unknown location; Bagru's stock check shows them as arriving without a document</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Confirm the courier codes: ATS = Amazon Shipping, XC = Xpressbees, DL / DLV / DE_* = Delhivery, BD_* = Blue Dart, EK_* = Ekart (all mapped from data evidence, unconfirmed).</t>
+          <t>Is the receiver the Bagru warehouse itself (stock coming back)? If yes, they are mapped to Bagru.</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -5687,102 +5840,8 @@
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>D-118</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>Inventory</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>Negative stock in the ERP report</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>Jaipur C-Scheme -10, Bangalore 7 -2 units</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>Stock totals slightly off; signals booking errors</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>An ERP glitch the ERP team cannot fix yet; the business is looking at it. 15 Sep 2026 report, sheet ChannelwiseStock: row 1602 coll003-1 Gift card at 08 Jaipur - C-Scheme -10; row 1673 GSTEA1905 at 29 FBA WH - Bangalore 7 -1; row 3030 SWETA2778 at 29 FBA WH - Bangalore 7 -1 (32 negative rows across the 19 reports). Decide: treat as 0, exclude, or show as reported (current).</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="inlineStr">
-        <is>
-          <t>Open - business</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="I43" s="4" t="inlineStr">
-        <is>
-          <t>ERP team</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>D-121</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>Purchase orders</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>PO lines with no due date</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>223 lines (3 still open)</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>Cannot be judged overdue</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>Fill due dates in the ERP (handled meanwhile: Schema 2.4: due_status 'No due date' on open PO lines)</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="inlineStr">
-        <is>
-          <t>Open - ERP team</t>
-        </is>
-      </c>
-      <c r="H44" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>ERP team</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I44"/>
+  <autoFilter ref="A1:I42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>